<commit_message>
feat: Stage 1 complete - rule-driven engineering platform
- Added Rules/ folder with thresholds, formulas, curves, constants (JSON)
- Integrated RuleEngine into pages 4,5,6,7,8
- Updated gt_performance.py and fuel_engine.py to use RuleEngine
- Deprecated corrections.py (replaced by RuleEngine)
- Updated constants.json with DECIMALS and other constants
- All pages now asset-agnostic (asset_type from session)
- Added Data/ folder for Excel files
- Removed config/ folder
- Updated excel_reader.py and unit_helpers.py
- Added docs/ folder with architecture markdown files
- Added check_rules.py and test_application.py for validation
- Updated requirements.txt with editable installs
- Fixed pyproject.toml for core and engineeros
</commit_message>
<xml_diff>
--- a/data/BASE LOAD PG TEST DATA 4 sets.xlsx
+++ b/data/BASE LOAD PG TEST DATA 4 sets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0696e3e181ec70ee/Documents/AI Projects/EngineeringPlatform/PlantIntelligencePlatform/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{2D0A8FA8-A8F1-F144-A402-B79B4DC5AF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F4C0CE7-7224-4E6D-B452-182AB8D7CF13}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="8_{2D0A8FA8-A8F1-F144-A402-B79B4DC5AF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59D3C34E-BE3A-4D0B-80FC-6E1E3F1143A7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -631,9 +631,6 @@
     <t>Unit</t>
   </si>
   <si>
-    <t xml:space="preserve">Tine </t>
-  </si>
-  <si>
     <t>PG TEST DATA</t>
   </si>
   <si>
@@ -650,6 +647,9 @@
   </si>
   <si>
     <t>Parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time </t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1073,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>199</v>
@@ -1082,19 +1082,19 @@
         <v>200</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>205</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -1121,7 +1121,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3748,6 +3748,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B16:E16"/>
@@ -3760,16 +3770,6 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>